<commit_message>
change folder structure at this pont we have chad,arch and value envoices
</commit_message>
<xml_diff>
--- a/Value/Value_MATERIAL_PRICES.xlsx
+++ b/Value/Value_MATERIAL_PRICES.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="3975" yWindow="1080" windowWidth="23340" windowHeight="12675" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="MATERIAL_MASTER" sheetId="1" state="visible" r:id="rId1"/>
@@ -28,8 +28,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy hh:mm"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -646,7 +647,7 @@
         </is>
       </c>
       <c r="J2" s="7" t="n">
-        <v>46287.3689308302</v>
+        <v>46287.38432890674</v>
       </c>
     </row>
     <row r="3">
@@ -679,7 +680,7 @@
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>46287.36893190214</v>
+        <v>46287.38432966034</v>
       </c>
     </row>
     <row r="4">
@@ -707,13 +708,13 @@
         <v>19.55</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" t="n">
-        <v>18.55</v>
+        <v>17.55</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>18.55</v>
+        <v>8.775</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
@@ -721,7 +722,7 @@
         </is>
       </c>
       <c r="J4" s="7" t="n">
-        <v>46287.36893126128</v>
+        <v>46287.38432920502</v>
       </c>
     </row>
     <row r="5">
@@ -754,7 +755,7 @@
         </is>
       </c>
       <c r="J5" s="7" t="n">
-        <v>46287.36893250645</v>
+        <v>46287.38433108568</v>
       </c>
     </row>
     <row r="6">
@@ -787,7 +788,7 @@
         </is>
       </c>
       <c r="J6" s="7" t="n">
-        <v>46287.36893250691</v>
+        <v>46287.3843310867</v>
       </c>
     </row>
     <row r="7">
@@ -820,7 +821,7 @@
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>46287.36893250727</v>
+        <v>46287.38433108697</v>
       </c>
     </row>
   </sheetData>
@@ -1036,7 +1037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1389,6 +1390,129 @@
         <v>34.24</v>
       </c>
       <c r="G11" t="inlineStr">
+        <is>
+          <t>Invoice_310189</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>KNAUF/EWI-100</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>100x1200x600mm Knauf EWI (24/p, 17.28m2)</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>19.55</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Invoice_308293</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>VOL/L44-100</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>100x1200x12000mm Easy Light 44 (14.4m2) 24/p</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>34.23</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Invoice_310189</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>VOL/L44-150</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>150x1200x8000mm Easy Light 44 (9.6m2) 24/p</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Invoice_310189</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>VOL/L44-200</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>200x1200x6000m Easy Light 44 (7.2m2) 24/p</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>Invoice_310189</t>
         </is>

</xml_diff>

<commit_message>
changed folder names and add Airpacks suplier pdf parsr logic also
</commit_message>
<xml_diff>
--- a/Value/Value_MATERIAL_PRICES.xlsx
+++ b/Value/Value_MATERIAL_PRICES.xlsx
@@ -28,9 +28,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/mm/yyyy hh:mm"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -551,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -646,8 +645,8 @@
           <t>311626</t>
         </is>
       </c>
-      <c r="J2" s="7" t="n">
-        <v>46287.38432890674</v>
+      <c r="J2" s="5" t="n">
+        <v>46287.38432891203</v>
       </c>
     </row>
     <row r="3">
@@ -680,7 +679,7 @@
         </is>
       </c>
       <c r="J3" s="7" t="n">
-        <v>46287.38432966034</v>
+        <v>46287.38881511294</v>
       </c>
     </row>
     <row r="4">
@@ -705,7 +704,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>19.55</v>
+        <v>30</v>
       </c>
       <c r="F4" t="n">
         <v>2</v>
@@ -721,8 +720,8 @@
           <t>Invoice_308293</t>
         </is>
       </c>
-      <c r="J4" s="7" t="n">
-        <v>46287.38432920502</v>
+      <c r="J4" s="5" t="n">
+        <v>46287.38432920139</v>
       </c>
     </row>
     <row r="5">
@@ -755,7 +754,7 @@
         </is>
       </c>
       <c r="J5" s="7" t="n">
-        <v>46287.38433108568</v>
+        <v>46287.38881547089</v>
       </c>
     </row>
     <row r="6">
@@ -782,13 +781,22 @@
       <c r="E6" t="n">
         <v>34.24</v>
       </c>
+      <c r="F6" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="G6" t="n">
+        <v>-2.73</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>-0.07384365701920476</v>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>Invoice_312384</t>
         </is>
       </c>
       <c r="J6" s="7" t="n">
-        <v>46287.3843310867</v>
+        <v>46287.38881547116</v>
       </c>
     </row>
     <row r="7">
@@ -815,13 +823,172 @@
       <c r="E7" t="n">
         <v>34.24</v>
       </c>
+      <c r="F7" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="G7" t="n">
+        <v>-2.73</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>-0.07384365701920476</v>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>Invoice_312384</t>
         </is>
       </c>
       <c r="J7" s="7" t="n">
-        <v>46287.38433108697</v>
+        <v>46287.38881547126</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>U/KNA/G/LR44-100</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Loft Roll 44 CombiCut 100mmx1140x1218 13.89m2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ROLL</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>33.06</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>9a56b318-cdc5-4bdb-914f-0a6befe846e5</t>
+        </is>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>46287.38881384544</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>U/KNA/G/LR44-150</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Loft Roll 44Combi Cut 150mm x1140x8050 9.18m2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ROLL</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>32.78</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>9a56b318-cdc5-4bdb-914f-0a6befe846e5</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>46287.3888138459</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>U/KNA/G/LR44-200</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Loft Roll(Combi Cut) 200mmx1140x6000 (6.84m2)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ROLL</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="F10" t="n">
+        <v>32.56</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>0.05159705159705159</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Invoice_306557</t>
+        </is>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>46287.38881440713</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RAV/120KG-120</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>120x600x1200mm EWI (2/pack) 120kg Pack</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>EACH</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>40.33</v>
+      </c>
+      <c r="F11" t="n">
+        <v>30</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>0.3443333333333333</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Invoice_304843 (1)</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>46287.3888141249</v>
       </c>
     </row>
   </sheetData>
@@ -1037,7 +1204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1513,6 +1680,720 @@
         <v>34.24</v>
       </c>
       <c r="G15" t="inlineStr">
+        <is>
+          <t>Invoice_310189</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>U/KNA/G/LR44-100</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Loft Roll 44 CombiCut 100mmx1140x1218 13.89m2</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>33.06</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>9a56b318-cdc5-4bdb-914f-0a6befe846e5</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>U/KNA/G/LR44-150</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Loft Roll 44Combi Cut 150mm x1140x8050 9.18m2</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>32.78</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>9a56b318-cdc5-4bdb-914f-0a6befe846e5</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>U/KNA/G/LR44-200</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Loft Roll(Combi Cut) 200mmx1140x6000 (6.84m2)</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>32.56</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>9a56b318-cdc5-4bdb-914f-0a6befe846e5</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>RAV/120KG-120</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>120x600x1200mm EWI (2/pack) 120kg Pack</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>40.33</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Invoice_304843 (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>U/KNA/G/LR44-200</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Loft Roll(Combi Cut) 200mmx1140x6000 (6.84m2)</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>32.56</v>
+      </c>
+      <c r="F20" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Invoice_306557</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>VOL/L44-150</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>150x1200x8000mm Easy Light 44 (9.6m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E21" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="F21" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Invoice_308294</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>VOL/L44-200</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>200x1200x6000m Easy Light 44 (7.2m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E22" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="F22" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Invoice_308294</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>VOL/L44-150</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>150x1200x8000mm Easy Light 44 (9.6m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="F23" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Invoice_310189</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>VOL/L44-200</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>200x1200x6000m Easy Light 44 (7.2m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="F24" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Invoice_310189</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>U/KNA/G/LR44-200</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Loft Roll(Combi Cut) 200mmx1140x6000 (6.84m2)</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="F25" t="n">
+        <v>32.56</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>9a56b318-cdc5-4bdb-914f-0a6befe846e5</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>U/KNA/G/LR44-200</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Loft Roll(Combi Cut) 200mmx1140x6000 (6.84m2)</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>32.56</v>
+      </c>
+      <c r="F26" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Invoice_306557</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>VOL/L44-150</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>150x1200x8000mm Easy Light 44 (9.6m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="F27" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Invoice_308294</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>VOL/L44-200</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>200x1200x6000m Easy Light 44 (7.2m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="F28" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Invoice_308294</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>VOL/L44-150</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>150x1200x8000mm Easy Light 44 (9.6m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="F29" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Invoice_310189</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>VOL/L44-200</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>200x1200x6000m Easy Light 44 (7.2m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E30" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="F30" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Invoice_310189</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>U/KNA/G/LR44-200</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Loft Roll(Combi Cut) 200mmx1140x6000 (6.84m2)</t>
+        </is>
+      </c>
+      <c r="E31" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="F31" t="n">
+        <v>32.56</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>9a56b318-cdc5-4bdb-914f-0a6befe846e5</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>RAV/120KG-120</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>120x600x1200mm EWI (2/pack) 120kg Pack</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>30</v>
+      </c>
+      <c r="F32" t="n">
+        <v>40.33</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Invoice_304843 (1)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>U/KNA/G/LR44-200</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Loft Roll(Combi Cut) 200mmx1140x6000 (6.84m2)</t>
+        </is>
+      </c>
+      <c r="E33" t="n">
+        <v>32.56</v>
+      </c>
+      <c r="F33" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Invoice_306557</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>VOL/L44-150</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>150x1200x8000mm Easy Light 44 (9.6m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E34" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="F34" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Invoice_308294</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>VOL/L44-200</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>200x1200x6000m Easy Light 44 (7.2m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="F35" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Invoice_308294</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>VOL/L44-150</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>150x1200x8000mm Easy Light 44 (9.6m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="F36" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Invoice_310189</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>22/09/2026</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>VOL/L44-200</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>200x1200x6000m Easy Light 44 (7.2m2) 24/p</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>36.97</v>
+      </c>
+      <c r="F37" t="n">
+        <v>34.24</v>
+      </c>
+      <c r="G37" t="inlineStr">
         <is>
           <t>Invoice_310189</t>
         </is>

</xml_diff>